<commit_message>
Add Purview classifier and workflow
</commit_message>
<xml_diff>
--- a/src/classifications/rajesh_delete.xlsx
+++ b/src/classifications/rajesh_delete.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wavicledata-my.sharepoint.com/personal/rajesh_puchakayala_wavicledata_com/Documents/Desktop/project/perview/classifications/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wavicledata-my.sharepoint.com/personal/rajesh_puchakayala_wavicledata_com/Documents/Desktop/project/perview/src/classifications/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="15" documentId="11_71F24F94407219B5A74575F6183D3E4314525CC4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C47B2A7A-D25E-4F3E-B568-441E396A51FA}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="14927" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="14927" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SQL Server" sheetId="1" r:id="rId1"/>
@@ -132,6 +132,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>